<commit_message>
- Introduced Invoice Date into excel as well
</commit_message>
<xml_diff>
--- a/src/main/resources/excel.xlsx
+++ b/src/main/resources/excel.xlsx
@@ -1,29 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20401"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saif.rehman\Desktop\murtaza\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\smsa\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A31DA096-E022-4377-A111-BF6B3A2B84EC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Account Number</t>
   </si>
@@ -59,15 +58,18 @@
   </si>
   <si>
     <t>Customer Name</t>
+  </si>
+  <si>
+    <t>Invoice Date</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="[$-409]dd\-mmm\-yy"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="[$-409]dd\-mmm\-yy"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -149,28 +151,28 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -183,7 +185,7 @@
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 3" xfId="2" xr:uid="{32A7960B-AC33-455E-866C-1E0BD411972B}"/>
+    <cellStyle name="Comma 3" xfId="2"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -396,73 +398,76 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.77734375" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.21875" style="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15" style="7" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.44140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.21875" style="7" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.77734375" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="22.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="23.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="12.6640625" style="6"/>
+    <col min="1" max="2" width="12.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" style="6" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.28515625" style="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" style="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="23.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="12.7109375" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>